<commit_message>
R2: Scenario A aligned (P&L revenue built from inputs), layer 2 group figures, ESCT brief; 36 of 36 pass live
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01MYp38cjP4DwiUggm3i2bkH
</commit_message>
<xml_diff>
--- a/docs/Audit/v6_0/smoke_test/3.1 Stress Test/scenario_a/review_scenario_a.xlsx
+++ b/docs/Audit/v6_0/smoke_test/3.1 Stress Test/scenario_a/review_scenario_a.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>157661</v>
+        <v>161710.69</v>
       </c>
     </row>
     <row r="11">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>59122.88</v>
+        <v>60641.51</v>
       </c>
     </row>
     <row r="12">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>157661</v>
+        <v>161710.69</v>
       </c>
     </row>
     <row r="15">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1011658.12</v>
+        <v>1015707.81</v>
       </c>
     </row>
     <row r="16">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1011658.12</v>
+        <v>1015707.81</v>
       </c>
     </row>
     <row r="19">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>102.2</v>
+        <v>102.61</v>
       </c>
     </row>
     <row r="22">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1313841.72</v>
+        <v>1347589.02</v>
       </c>
     </row>
     <row r="23">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>197076.26</v>
+        <v>202138.35</v>
       </c>
     </row>
     <row r="24">
@@ -680,101 +680,283 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1116765.46</v>
+        <v>1145450.67</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>business_outcome.group.da376b9f-9af9-5956-ae1e-5845c3fc367f.modelled_revenue</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>233329.25</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>P&amp;L summary</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr"/>
+          <t>business_outcome.group.da376b9f-9af9-5956-ae1e-5845c3fc367f.capacity_gap_hours</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>265.88</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>revenue</t>
+          <t>cost_allocation.group.da376b9f-9af9-5956-ae1e-5845c3fc367f.idle_labour_hours</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1313841.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>labour_lines</t>
+          <t>cost_allocation.group.da376b9f-9af9-5956-ae1e-5845c3fc367f.idle_labour_cost</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>812167.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>asset_interest</t>
+          <t>business_outcome.group.da376b9f-9af9-5956-ae1e-5845c3fc367f.capacity_gap_dollars</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>41829.83</v>
+        <v>43870.75</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>net_profit</t>
+          <t>business_outcome.group.8eb72391-aa1b-58ff-add5-2fa40b343cb2.modelled_revenue</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>105107.34</v>
+        <v>341400</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>business_outcome.group.8eb72391-aa1b-58ff-add5-2fa40b343cb2.capacity_gap_hours</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>-163.23</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Charge-out per staff type</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr"/>
+          <t>cost_allocation.group.8eb72391-aa1b-58ff-add5-2fa40b343cb2.idle_labour_hours</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>163.23</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>operator_delivery_staff</t>
+          <t>cost_allocation.group.8eb72391-aa1b-58ff-add5-2fa40b343cb2.idle_labour_cost</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>90</v>
+        <v>9414.83</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>senior_operator_staff</t>
+          <t>business_outcome.group.8eb72391-aa1b-58ff-add5-2fa40b343cb2.capacity_gap_dollars</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>105</v>
+        <v>9414.83</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>business_outcome.group.343523b7-f1e2-5676-a399-e165670f7a19.modelled_revenue</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>226258.67</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>business_outcome.group.343523b7-f1e2-5676-a399-e165670f7a19.capacity_gap_hours</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>265.88</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>cost_allocation.group.343523b7-f1e2-5676-a399-e165670f7a19.idle_labour_hours</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>cost_allocation.group.343523b7-f1e2-5676-a399-e165670f7a19.idle_labour_cost</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>business_outcome.group.343523b7-f1e2-5676-a399-e165670f7a19.capacity_gap_dollars</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>42541.33</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>business_outcome.group.ee8a6818-a0a0-53ad-a202-900b55035375.modelled_revenue</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>304035.08</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>P&amp;L summary</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>revenue_basis</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>billed_from_rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>billed_from_rates</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1105023</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1347589.02</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>labour_lines</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>812167.28</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>asset_interest</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>41829.83</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>net_profit</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>129742.86</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Charge-out per staff type</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>operator_delivery_staff</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>senior_operator_staff</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
           <t>supervisor_team_lead</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
-        <v>120</v>
+      <c r="B53" s="5" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2110,7 +2292,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="5" t="n">
-        <v>1313841.72</v>
+        <v>1347589.02</v>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
@@ -2140,7 +2322,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>197076.26</v>
+        <v>202138.35</v>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
@@ -2260,7 +2442,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>32846.04</v>
+        <v>33689.73</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
@@ -2290,7 +2472,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>19707.63</v>
+        <v>20213.84</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
@@ -2320,7 +2502,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>10510.73</v>
+        <v>10780.71</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
@@ -2350,7 +2532,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>7883.05</v>
+        <v>8085.53</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
@@ -2380,7 +2562,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>6569.21</v>
+        <v>6737.95</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
@@ -2410,7 +2592,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>10510.73</v>
+        <v>10780.71</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
@@ -2440,7 +2622,7 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>10510.73</v>
+        <v>10780.71</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
@@ -2470,7 +2652,7 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>39415.25</v>
+        <v>40427.67</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
@@ -2500,7 +2682,7 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>19707.63</v>
+        <v>20213.84</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
@@ -2603,7 +2785,7 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>1</v>
@@ -2626,7 +2808,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>1</v>
@@ -2649,7 +2831,7 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>1</v>
@@ -2672,7 +2854,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>1</v>

</xml_diff>